<commit_message>
Daily slate 2026-06-19 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-17.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-17.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="E4" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F4" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G4" t="n">
-        <v>54.1</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="5">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E7" t="n">
         <v>54</v>
       </c>
       <c r="F7" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G7" t="n">
-        <v>61.4</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E9" t="n">
         <v>30</v>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G9" t="n">
-        <v>54.5</v>
+        <v>53.6</v>
       </c>
     </row>
     <row r="10">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1150</v>
+        <v>1173</v>
       </c>
       <c r="E11" t="n">
-        <v>757</v>
+        <v>767</v>
       </c>
       <c r="F11" t="n">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="G11" t="n">
-        <v>65.8</v>
+        <v>65.40000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="E12" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="F12" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G12" t="n">
-        <v>67.2</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="E14" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F14" t="n">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="G14" t="n">
-        <v>27.7</v>
+        <v>27.3</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>589</v>
+        <v>601</v>
       </c>
       <c r="E15" t="n">
         <v>112</v>
       </c>
       <c r="F15" t="n">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="G15" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E16" t="n">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F16" t="n">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="G16" t="n">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4388</v>
+        <v>4505</v>
       </c>
       <c r="E17" t="n">
-        <v>1014</v>
+        <v>1030</v>
       </c>
       <c r="F17" t="n">
-        <v>3374</v>
+        <v>3475</v>
       </c>
       <c r="G17" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
     </row>
   </sheetData>
@@ -1427,7 +1427,7 @@
         <v>51</v>
       </c>
       <c r="N5" t="n">
-        <v>28.9</v>
+        <v>27.8</v>
       </c>
       <c r="O5" t="n">
         <v>90</v>
@@ -1582,16 +1582,16 @@
         <v>335</v>
       </c>
       <c r="D7" t="n">
-        <v>65.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>1150</v>
+        <v>1173</v>
       </c>
       <c r="F7" t="n">
-        <v>67.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="H7" t="n">
         <v>42</v>
@@ -1600,28 +1600,28 @@
         <v>162</v>
       </c>
       <c r="J7" t="n">
-        <v>27.7</v>
+        <v>27.3</v>
       </c>
       <c r="K7" t="n">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="L7" t="n">
-        <v>19</v>
+        <v>18.6</v>
       </c>
       <c r="M7" t="n">
-        <v>589</v>
+        <v>601</v>
       </c>
       <c r="N7" t="n">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
       <c r="O7" t="n">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="P7" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>4388</v>
+        <v>4505</v>
       </c>
       <c r="R7" t="n">
         <v>54.4</v>
@@ -1630,10 +1630,10 @@
         <v>428</v>
       </c>
       <c r="T7" t="n">
-        <v>54.1</v>
+        <v>53.2</v>
       </c>
       <c r="U7" t="n">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
@@ -1660,16 +1660,16 @@
         <v>105</v>
       </c>
       <c r="AD7" t="n">
-        <v>61.4</v>
+        <v>60</v>
       </c>
       <c r="AE7" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AF7" t="n">
-        <v>54.5</v>
+        <v>53.6</v>
       </c>
       <c r="AG7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-06-20 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-17.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-17.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>156</v>
+        <v>397</v>
       </c>
       <c r="E4" t="n">
-        <v>83</v>
+        <v>161</v>
       </c>
       <c r="F4" t="n">
-        <v>73</v>
+        <v>236</v>
       </c>
       <c r="G4" t="n">
-        <v>53.2</v>
+        <v>40.6</v>
       </c>
     </row>
     <row r="5">
@@ -587,13 +587,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="E8" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="G8" t="n">
-        <v>54.9</v>
+        <v>41.3</v>
       </c>
     </row>
     <row r="9">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>335</v>
+        <v>518</v>
       </c>
       <c r="E10" t="n">
-        <v>217</v>
+        <v>256</v>
       </c>
       <c r="F10" t="n">
-        <v>118</v>
+        <v>262</v>
       </c>
       <c r="G10" t="n">
-        <v>64.8</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="11">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4505</v>
+        <v>5339</v>
       </c>
       <c r="E17" t="n">
-        <v>1030</v>
+        <v>1115</v>
       </c>
       <c r="F17" t="n">
-        <v>3475</v>
+        <v>4224</v>
       </c>
       <c r="G17" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
     </row>
   </sheetData>
@@ -1297,10 +1297,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60.4</v>
+        <v>29.4</v>
       </c>
       <c r="C4" t="n">
-        <v>48</v>
+        <v>231</v>
       </c>
       <c r="D4" t="n">
         <v>51.3</v>
@@ -1339,10 +1339,10 @@
         <v>78</v>
       </c>
       <c r="P4" t="n">
-        <v>9.6</v>
+        <v>10.1</v>
       </c>
       <c r="Q4" t="n">
-        <v>73</v>
+        <v>907</v>
       </c>
       <c r="R4" t="n">
         <v>50.9</v>
@@ -1351,19 +1351,22 @@
         <v>55</v>
       </c>
       <c r="T4" t="n">
-        <v>100</v>
+        <v>32.9</v>
       </c>
       <c r="U4" t="n">
-        <v>2</v>
+        <v>243</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="X4" t="n">
-        <v>54.5</v>
+        <v>32.8</v>
       </c>
       <c r="Y4" t="n">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="Z4" t="n">
         <v>53.8</v>
@@ -1576,10 +1579,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>64.8</v>
+        <v>49.4</v>
       </c>
       <c r="C7" t="n">
-        <v>335</v>
+        <v>518</v>
       </c>
       <c r="D7" t="n">
         <v>65.40000000000001</v>
@@ -1618,10 +1621,10 @@
         <v>475</v>
       </c>
       <c r="P7" t="n">
-        <v>22.9</v>
+        <v>20.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>4505</v>
+        <v>5339</v>
       </c>
       <c r="R7" t="n">
         <v>54.4</v>
@@ -1630,22 +1633,22 @@
         <v>428</v>
       </c>
       <c r="T7" t="n">
-        <v>53.2</v>
+        <v>40.6</v>
       </c>
       <c r="U7" t="n">
-        <v>156</v>
+        <v>397</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X7" t="n">
-        <v>54.9</v>
+        <v>41.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="Z7" t="n">
         <v>58</v>

</xml_diff>